<commit_message>
Changes made in DB classes
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/ScenarioDetails.xlsx
+++ b/src/test/resources/TestData/ScenarioDetails.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
   <si>
     <t xml:space="preserve">testScenarioID</t>
   </si>
@@ -31,6 +31,18 @@
     <t xml:space="preserve">testEnabled</t>
   </si>
   <si>
+    <t xml:space="preserve">FeatureName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SmokeSuite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RegressionSuite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parallel Mode</t>
+  </si>
+  <si>
     <t xml:space="preserve">testScenarioID1</t>
   </si>
   <si>
@@ -40,25 +52,34 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
+    <t xml:space="preserve">Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">testScenarioID2</t>
   </si>
   <si>
     <t xml:space="preserve">testScenarioName2</t>
   </si>
   <si>
+    <t xml:space="preserve">Dashboard</t>
+  </si>
+  <si>
     <t xml:space="preserve">testScenarioID3</t>
   </si>
   <si>
     <t xml:space="preserve">testScenarioName3</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
     <t xml:space="preserve">testScenarioID4</t>
   </si>
   <si>
     <t xml:space="preserve">testScenarioName4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuiteType=Smoke,Regression</t>
   </si>
 </sst>
 </file>
@@ -73,6 +94,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -95,6 +117,7 @@
       <color rgb="FF000000"/>
       <name val="Menlo"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -165,11 +188,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="28.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="28.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -182,49 +207,114 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="0" t="s">
         <v>10</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D10" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>